<commit_message>
Match monthly files' print setup: A4, margins, page footer
Re-export PDF from the workbook so the PDF matches the Excel print.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013iJC5cHDg1h7fwyet2RwNx
</commit_message>
<xml_diff>
--- a/Faiz_Patient_Data_Master_Nov2025-Oct2026.xlsx
+++ b/Faiz_Patient_Data_Master_Nov2025-Oct2026.xlsx
@@ -4546,11 +4546,11 @@
     <hyperlink ref="B15" r:id="rId12" location="'Oct-2026'!A1" display="October 2026"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="true" verticalCentered="false"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.511811023622047" footer="0.5"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
-    <oddFooter/>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;9 Page &amp;P of &amp;N</oddFooter>
   </headerFooter>
 </worksheet>
 </file>
@@ -4772,11 +4772,11 @@
     <mergeCell ref="A25:D25"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="true" verticalCentered="false"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.511811023622047" footer="0.5"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
-    <oddFooter/>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;9 Page &amp;P of &amp;N</oddFooter>
   </headerFooter>
 </worksheet>
 </file>
@@ -6374,11 +6374,11 @@
     <mergeCell ref="A95:D95"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="true" verticalCentered="false"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.511811023622047" footer="0.5"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
-    <oddFooter/>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;9 Page &amp;P of &amp;N</oddFooter>
   </headerFooter>
 </worksheet>
 </file>
@@ -7138,11 +7138,11 @@
     <mergeCell ref="A45:D45"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="true" verticalCentered="false"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.511811023622047" footer="0.5"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
-    <oddFooter/>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;9 Page &amp;P of &amp;N</oddFooter>
   </headerFooter>
 </worksheet>
 </file>
@@ -7598,11 +7598,11 @@
     <mergeCell ref="A27:D27"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="true" verticalCentered="false"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.511811023622047" footer="0.5"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
-    <oddFooter/>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;9 Page &amp;P of &amp;N</oddFooter>
   </headerFooter>
 </worksheet>
 </file>
@@ -7769,11 +7769,11 @@
     <mergeCell ref="A10:D10"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="true" verticalCentered="false"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.511811023622047" footer="0.5"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
-    <oddFooter/>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;9 Page &amp;P of &amp;N</oddFooter>
   </headerFooter>
 </worksheet>
 </file>
@@ -9419,11 +9419,11 @@
     <mergeCell ref="A97:D97"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="true" verticalCentered="false"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.511811023622047" footer="0.5"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
-    <oddFooter/>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;9 Page &amp;P of &amp;N</oddFooter>
   </headerFooter>
 </worksheet>
 </file>
@@ -10373,11 +10373,11 @@
     <mergeCell ref="A57:D57"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="true" verticalCentered="false"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.511811023622047" footer="0.5"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
-    <oddFooter/>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;9 Page &amp;P of &amp;N</oddFooter>
   </headerFooter>
 </worksheet>
 </file>
@@ -12710,11 +12710,11 @@
     <mergeCell ref="A140:D140"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="true" verticalCentered="false"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.511811023622047" footer="0.5"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
-    <oddFooter/>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;9 Page &amp;P of &amp;N</oddFooter>
   </headerFooter>
 </worksheet>
 </file>
@@ -13812,11 +13812,11 @@
     <mergeCell ref="A65:D65"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="true" verticalCentered="false"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.511811023622047" footer="0.5"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
-    <oddFooter/>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;9 Page &amp;P of &amp;N</oddFooter>
   </headerFooter>
 </worksheet>
 </file>
@@ -14959,11 +14959,11 @@
     <mergeCell ref="A68:D68"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="true" verticalCentered="false"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.511811023622047" footer="0.5"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
-    <oddFooter/>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;9 Page &amp;P of &amp;N</oddFooter>
   </headerFooter>
 </worksheet>
 </file>
@@ -15883,11 +15883,11 @@
     <mergeCell ref="A57:D57"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="true" verticalCentered="false"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.511811023622047" footer="0.5"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
-    <oddFooter/>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;9 Page &amp;P of &amp;N</oddFooter>
   </headerFooter>
 </worksheet>
 </file>
@@ -16864,11 +16864,11 @@
     <mergeCell ref="A58:D58"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="true" verticalCentered="false"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.511811023622047" footer="0.5"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
-    <oddFooter/>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;9 Page &amp;P of &amp;N</oddFooter>
   </headerFooter>
 </worksheet>
 </file>
</xml_diff>